<commit_message>
data de revisão do modelo de solda
</commit_message>
<xml_diff>
--- a/modelo_op_solda.xlsx
+++ b/modelo_op_solda.xlsx
@@ -23,8 +23,8 @@
 Página</t>
   </si>
   <si>
-    <t>RQ PCP-016-000
-02/01/2024
+    <t>RQ PCP-030-000
+22/04/2025
 -
 N/A</t>
   </si>
@@ -510,7 +510,7 @@
       <alignment horizontal="left" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="6" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="top" wrapText="1"/>
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="7" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyFont="1"/>

</xml_diff>